<commit_message>
feat(valuation-parser): complete Phase 4 with enhanced review and routing logic
- Added review item generation for valuation subjects
- Improved routing logic to handle edge cases in custodian mapping
- Validated outputs with output_phase4 directory
- Updated parse_summary.md and eview_items.csv for Phase 4
- Enhanced test coverage for review and routing modules
</commit_message>
<xml_diff>
--- a/data_samples/raw/估值表日报-XXX022-PRODUCT_022-4-20250327.xlsx
+++ b/data_samples/raw/估值表日报-XXX022-PRODUCT_022-4-20250327.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x15">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <ns1:AlternateContent>
-    <ns1:Choice Requires="x15">
-      <ns2:absPath url="D:\估值V2.6\Management\06常用工具\95微服务自动导出报表\Release\Sources\Trunk\fa-report-service\report\Public\AccountValuate\templet\"/>
-    </ns1:Choice>
-  </ns1:AlternateContent>
+  <mc:AlternateContent>
+    <mc:Choice Requires="x15">
+      <x15ac:absPath url="D:\估值V2.6\Management\06常用工具\95微服务自动导出报表\Release\Sources\Trunk\fa-report-service\report\Public\AccountValuate\templet\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28125" windowHeight="12540"/>
   </bookViews>
@@ -2971,12 +2971,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:K137"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" ns2:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="23.625" collapsed="false"/>
     <col min="2" max="2" customWidth="true" style="1" width="23.875" collapsed="false"/>
@@ -2989,7 +2989,7 @@
     <col min="9" max="11" customWidth="true" width="21.875" collapsed="false"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="25.5" ns2:dyDescent="0.15">
+    <row r="1" spans="1:11" ht="25.5" x14ac:dyDescent="0.15">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -3004,7 +3004,7 @@
       <c r="J1" s="24"/>
       <c r="K1"/>
     </row>
-    <row r="2" spans="1:11" ns2:dyDescent="0.15">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A2" s="25" t="s">
         <v>226</v>
       </c>
@@ -3019,7 +3019,7 @@
       <c r="J2" s="25"/>
       <c r="K2"/>
     </row>
-    <row r="3" spans="1:11" ns2:dyDescent="0.15">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A3" s="26" t="s">
         <v>228</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="22.5" customHeight="1" ns2:dyDescent="0.15">
+    <row r="4" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>4</v>
       </c>
@@ -3073,7 +3073,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ns2:dyDescent="0.15">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A5" s="52" t="s">
         <v>68</v>
       </c>
@@ -3100,7 +3100,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ns2:dyDescent="0.15" ht="13.5" customHeight="true">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.15" ht="13.5" customHeight="true">
       <c r="A6" s="15" t="s">
         <v>70</v>
       </c>
@@ -3127,7 +3127,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ns2:dyDescent="0.15" ht="13.5" customHeight="true">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.15" ht="13.5" customHeight="true">
       <c r="A7" s="15" t="s">
         <v>72</v>
       </c>

</xml_diff>